<commit_message>
Checkpoint r6 combat audit: 40 reviewed abilities and historical settlement fixes
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="Rbd2373f7faba45a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="Ra9c4f20d07c44037"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R0cb977b356304b0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R9838eb0380f942bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R25124035d7724076"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="Rce6adc72d7074f4e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -161,7 +161,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Config_units_2" displayName="Config_units_2" ref="A4:F54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Config_units_2" displayName="Config_units_2" ref="A4:F55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="组"/>
     <x:tableColumn id="2" name="字段"/>
@@ -701,7 +701,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8af623e8bcda4763"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfde1396245a24777"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1455,7 +1455,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3e1cb43e8ec4ca1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4da3d561db3849ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2505,10 +2505,30 @@
         <x:v>现有EXTRA_WORKING_DEFAULTS工作数值，未声称Dota核验</x:v>
       </x:c>
     </x:row>
+    <x:row r="55" ht="60" customHeight="1">
+      <x:c r="A55" s="8" t="str">
+        <x:v>battle</x:v>
+      </x:c>
+      <x:c r="B55" s="8" t="str">
+        <x:v>spellLifestealCreepFactor</x:v>
+      </x:c>
+      <x:c r="C55" s="8" t="str">
+        <x:v>技能吸血对普通非英雄单位的倍率</x:v>
+      </x:c>
+      <x:c r="D55" s="9" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="E55" s="8" t="str">
+        <x:v>倍率</x:v>
+      </x:c>
+      <x:c r="F55" s="8" t="str">
+        <x:v>2022-2023历史Spell Lifesteal：普通非英雄仅20%，幻象与类英雄另行判定；不扩大为所有summoned单位。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc453040183304d23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd881fae38c27493f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint r6 C4: native attack profiles, 65 reviewed skills and startup phases
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R9838eb0380f942bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R25124035d7724076"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="Rce6adc72d7074f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R1860e818d0c6409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R1d561178daf149ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R6da8376c68e14a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R4b613c06053247b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="General"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -46,7 +48,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -63,6 +65,11 @@
         <x:fgColor rgb="FFFFF4D0"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B63"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -76,7 +83,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -98,6 +105,20 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -134,8 +155,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Config_units_1" displayName="Config_units_1" ref="A4:S15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="19">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Config_units_1" displayName="Config_units_1" ref="A4:T17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="20">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
     <x:tableColumn id="3" name="生命"/>
@@ -155,13 +176,14 @@
     <x:tableColumn id="17" name="转身速度rad每秒"/>
     <x:tableColumn id="18" name="弹体速度"/>
     <x:tableColumn id="19" name="攻击距离缓冲"/>
+    <x:tableColumn id="20" name="攻击类型0无1近2远"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Config_units_2" displayName="Config_units_2" ref="A4:F55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Config_units_2" displayName="Config_units_2" ref="A4:F56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="组"/>
     <x:tableColumn id="2" name="字段"/>
@@ -169,6 +191,17 @@
     <x:tableColumn id="4" name="数值"/>
     <x:tableColumn id="5" name="单位"/>
     <x:tableColumn id="6" name="来源说明"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="单位ID"/>
+    <x:tableColumn id="2" name="来源"/>
+    <x:tableColumn id="3" name="冲突或换算说明"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -701,7 +734,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfde1396245a24777"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0be7cedbdf064bd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -732,6 +765,7 @@
     <x:col min="17" max="17" width="17" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="17" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -741,7 +775,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>固定Valve 2023-02-10候选模板。AA技能明确生命/攻击等优先；随施法者变化的系数维护在技能表。未提供的转身与后摇为项目工作值。</x:v>
+        <x:v>原生模板数值：基础攻击间隔与基础攻速独立；攻击类型0无/1近战/2远程。时序/弹速/转身来源及冲突裁决见“原生单位来源”。四职业平衡不受本表校准影响。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
@@ -802,6 +836,9 @@
       <x:c r="S4" s="7" t="str">
         <x:v>攻击距离缓冲</x:v>
       </x:c>
+      <x:c r="T4" s="7" t="str">
+        <x:v>攻击类型0无1近2远</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="8" t="str">
@@ -853,13 +890,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q5" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="R5" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="S5" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T5" s="10" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -897,7 +937,7 @@
         <x:v>467</x:v>
       </x:c>
       <x:c r="L6" s="9" t="n">
-        <x:v>1133</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="M6" s="9" t="n">
         <x:v>100</x:v>
@@ -912,13 +952,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q6" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>16.666666666666668</x:v>
       </x:c>
       <x:c r="R6" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="S6" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T6" s="10" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
@@ -956,7 +999,7 @@
         <x:v>467</x:v>
       </x:c>
       <x:c r="L7" s="9" t="n">
-        <x:v>932.9999999999998</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="M7" s="9" t="n">
         <x:v>100</x:v>
@@ -971,13 +1014,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q7" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>16.666666666666668</x:v>
       </x:c>
       <x:c r="R7" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="S7" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T7" s="10" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
@@ -1015,7 +1061,7 @@
         <x:v>330</x:v>
       </x:c>
       <x:c r="L8" s="9" t="n">
-        <x:v>570.0000000000001</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="M8" s="9" t="n">
         <x:v>90</x:v>
@@ -1030,13 +1076,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q8" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>16.666666666666668</x:v>
       </x:c>
       <x:c r="R8" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="S8" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T8" s="10" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
@@ -1071,10 +1120,10 @@
         <x:v>109</x:v>
       </x:c>
       <x:c r="K9" s="9" t="n">
-        <x:v>275.2293577981651</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="L9" s="9" t="n">
-        <x:v>642.2018348623852</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="M9" s="9" t="n">
         <x:v>550</x:v>
@@ -1089,13 +1138,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q9" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>16.666666666666668</x:v>
       </x:c>
       <x:c r="R9" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="S9" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T9" s="10" t="n">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
@@ -1130,10 +1182,10 @@
         <x:v>109</x:v>
       </x:c>
       <x:c r="K10" s="9" t="n">
-        <x:v>206.42201834862385</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="L10" s="9" t="n">
-        <x:v>481.651376146789</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="M10" s="9" t="n">
         <x:v>100</x:v>
@@ -1148,13 +1200,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q10" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>16.666666666666668</x:v>
       </x:c>
       <x:c r="R10" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="S10" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T10" s="10" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
@@ -1189,10 +1244,10 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="K11" s="9" t="n">
-        <x:v>400</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="L11" s="9" t="n">
-        <x:v>1266.6666666666665</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="M11" s="9" t="n">
         <x:v>300</x:v>
@@ -1207,13 +1262,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="Q11" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>30.000000000000004</x:v>
       </x:c>
       <x:c r="R11" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="S11" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T11" s="10" t="n">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
@@ -1248,10 +1306,10 @@
         <x:v>135</x:v>
       </x:c>
       <x:c r="K12" s="9" t="n">
-        <x:v>400</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="L12" s="9" t="n">
-        <x:v>1081.4814814814815</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="M12" s="9" t="n">
         <x:v>300</x:v>
@@ -1266,13 +1324,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="Q12" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>30.000000000000004</x:v>
       </x:c>
       <x:c r="R12" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="S12" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T12" s="10" t="n">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
@@ -1307,10 +1368,10 @@
         <x:v>150</x:v>
       </x:c>
       <x:c r="K13" s="9" t="n">
-        <x:v>399.99999999999994</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="L13" s="9" t="n">
-        <x:v>933.3333333333334</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="M13" s="9" t="n">
         <x:v>128</x:v>
@@ -1325,13 +1386,16 @@
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="Q13" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>16.666666666666668</x:v>
       </x:c>
       <x:c r="R13" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="S13" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T13" s="10" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
@@ -1369,7 +1433,7 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="L14" s="9" t="n">
-        <x:v>1033.3333333333333</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="M14" s="9" t="n">
         <x:v>100</x:v>
@@ -1384,13 +1448,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="Q14" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>30.000000000000004</x:v>
       </x:c>
       <x:c r="R14" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="S14" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T14" s="10" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
@@ -1428,7 +1495,7 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="L15" s="9" t="n">
-        <x:v>1033.3333333333333</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="M15" s="9" t="n">
         <x:v>100</x:v>
@@ -1443,19 +1510,146 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="Q15" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>16.666666666666668</x:v>
       </x:c>
       <x:c r="R15" s="9" t="n">
-        <x:v>1400</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="S15" s="9" t="n">
-        <x:v>50</x:v>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T15" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="8" t="str">
+        <x:v>npc_dota_witch_doctor_death_ward</x:v>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
+        <x:v>死亡守卫</x:v>
+      </x:c>
+      <x:c r="C16" s="9" t="n">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="D16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" s="9" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="J16" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M16" s="9" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="N16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O16" s="9" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="P16" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q16" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R16" s="9" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S16" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T16" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="8" t="str">
+        <x:v>npc_dota_lich_ice_spire</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>冰柱</x:v>
+      </x:c>
+      <x:c r="C17" s="9" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="9" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="J17" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q17" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R17" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S17" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T17" s="10" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4da3d561db3849ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdde18527466d4d9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2525,10 +2719,211 @@
         <x:v>2022-2023历史Spell Lifesteal：普通非英雄仅20%，幻象与类英雄另行判定；不扩大为所有summoned单位。</x:v>
       </x:c>
     </x:row>
+    <x:row r="56" ht="80" customHeight="1">
+      <x:c r="A56" s="8" t="str">
+        <x:v>battle</x:v>
+      </x:c>
+      <x:c r="B56" s="8" t="str">
+        <x:v>baseManaRegen</x:v>
+      </x:c>
+      <x:c r="C56" s="8" t="str">
+        <x:v>基础每秒法力恢复</x:v>
+      </x:c>
+      <x:c r="D56" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E56" s="8" t="str">
+        <x:v>法力/秒</x:v>
+      </x:c>
+      <x:c r="F56" s="15" t="str">
+        <x:v>原工程固定3点/秒迁入配置，不冒称原生Dota数值；native召唤物以StatusManaRegen减去此基础恢复，保持自身原生速率。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd881fae38c27493f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7991a737ce434fbe"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="52" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="110" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="110" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>原生单位攻击与移动配置来源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>数值权威在“召唤单位”；本页仅说明来源与候选换算，不提供另一份可编辑副本。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="26" customHeight="1">
+      <x:c r="A4" s="12" t="str">
+        <x:v>单位ID</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>来源</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>冲突或换算说明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="64" customHeight="1">
+      <x:c r="A5" s="14" t="str">
+        <x:v>npc_dota_beastmaster_hawk_4</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>https://web.archive.org/web/20230215191303id_/https://dota2.fandom.com/wiki/Beastmaster</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.6；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="14" t="str">
+        <x:v>npc_dota_furion_treant_4</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="str">
+        <x:v>https://web.archive.org/web/20230215192014id_/https://dota2.fandom.com/wiki/Nature's_Prophet</x:v>
+      </x:c>
+      <x:c r="C6" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。树人KV2.5与Wiki0.5冲突，采用Wiki。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="14" t="str">
+        <x:v>npc_dota_furion_treant_large</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str">
+        <x:v>https://liquipedia.net/dota2/Greater_Treant_%287.28-7.31d%29</x:v>
+      </x:c>
+      <x:c r="C7" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。树人KV2.5与Wiki0.5冲突，采用Wiki。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="64" customHeight="1">
+      <x:c r="A8" s="14" t="str">
+        <x:v>npc_dota_lycan_wolf4</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>https://web.archive.org/web/20230205103458id_/https://dota2.fandom.com/wiki/Lycan</x:v>
+      </x:c>
+      <x:c r="C8" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
+      <x:c r="A9" s="14" t="str">
+        <x:v>npc_dota_necronomicon_archer_3</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>https://web.archive.org/web/20230215203000id_/https://dota2.fandom.com/wiki/Necronomicon</x:v>
+      </x:c>
+      <x:c r="C9" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="64" customHeight="1">
+      <x:c r="A10" s="14" t="str">
+        <x:v>npc_dota_necronomicon_warrior_3</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>https://web.archive.org/web/20230215203000id_/https://dota2.fandom.com/wiki/Necronomicon</x:v>
+      </x:c>
+      <x:c r="C10" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="64" customHeight="1">
+      <x:c r="A11" s="14" t="str">
+        <x:v>npc_dota_neutral_big_thunder_lizard</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str">
+        <x:v>https://web.archive.org/web/20220927090953id_/https://dota2.fandom.com/wiki/Ancient_Thunderhide</x:v>
+      </x:c>
+      <x:c r="C11" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.9；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="64" customHeight="1">
+      <x:c r="A12" s="14" t="str">
+        <x:v>npc_dota_neutral_black_dragon</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>https://web.archive.org/web/20230227161557id_/https://dota2.fandom.com/wiki/Ancient_Black_Dragon</x:v>
+      </x:c>
+      <x:c r="C12" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.9；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="64" customHeight="1">
+      <x:c r="A13" s="14" t="str">
+        <x:v>npc_dota_neutral_granite_golem</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="str">
+        <x:v>https://web.archive.org/web/20220701112441id_/https://dota2.fandom.com/wiki/Ancient_Granite_Golem</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="64" customHeight="1">
+      <x:c r="A14" s="14" t="str">
+        <x:v>npc_dota_neutral_mud_golem</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="str">
+        <x:v>https://web.archive.org/web/20221205165935id_/https://dota2.fandom.com/wiki/Mud_Golem</x:v>
+      </x:c>
+      <x:c r="C14" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.9；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。泥土傀儡KV继承0.5与Wiki0.9冲突，采用Wiki。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="64" customHeight="1">
+      <x:c r="A15" s="14" t="str">
+        <x:v>npc_dota_neutral_mud_golem_split</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>https://web.archive.org/web/20220707081432id_/https://dota2.fandom.com/wiki/Shard_Golem</x:v>
+      </x:c>
+      <x:c r="C15" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="64" customHeight="1">
+      <x:c r="A16" s="14" t="str">
+        <x:v>npc_dota_witch_doctor_death_ward</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="str">
+        <x:v>https://web.archive.org/web/20230215192255id_/https://dota2.fandom.com/wiki/Witch_Doctor</x:v>
+      </x:c>
+      <x:c r="C16" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="64" customHeight="1">
+      <x:c r="A17" s="14" t="str">
+        <x:v>npc_dota_lich_ice_spire</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="str">
+        <x:v>references/dota-20230216/parsed/npc_units.json</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="str">
+        <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。基础攻速100、后摇0为缺省候选；无攻击能力使攻击时钟无效。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11ce1bb33d154360"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint r6 C7: attack composition, frost control and 110 reviewed skills
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R1860e818d0c6409c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R1d561178daf149ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R6da8376c68e14a16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R4b613c06053247b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="Rb5b19717e0604f7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R1791269c7982447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R00fe29731cf94c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="Ra667aeb5d1e94c62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,8 +155,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Config_units_1" displayName="Config_units_1" ref="A4:T17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="20">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:U18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="21">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
     <x:tableColumn id="3" name="生命"/>
@@ -177,6 +177,7 @@
     <x:tableColumn id="18" name="弹体速度"/>
     <x:tableColumn id="19" name="攻击距离缓冲"/>
     <x:tableColumn id="20" name="攻击类型0无1近2远"/>
+    <x:tableColumn id="21" name="原生等级"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -197,7 +198,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>
@@ -734,7 +735,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0be7cedbdf064bd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59d2010013514261"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -766,6 +767,7 @@
     <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="17" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="22" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -839,6 +841,9 @@
       <x:c r="T4" s="7" t="str">
         <x:v>攻击类型0无1近2远</x:v>
       </x:c>
+      <x:c r="U4" s="7" t="str">
+        <x:v>原生等级</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="8" t="str">
@@ -901,6 +906,9 @@
       <x:c r="T5" s="10" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="U5" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
       <x:c r="A6" s="8" t="str">
@@ -963,6 +971,9 @@
       <x:c r="T6" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U6" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="8" t="str">
@@ -1025,6 +1036,9 @@
       <x:c r="T7" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U7" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="8" t="str">
@@ -1087,6 +1101,9 @@
       <x:c r="T8" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U8" s="10" t="n">
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="8" t="str">
@@ -1149,6 +1166,9 @@
       <x:c r="T9" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U9" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="8" t="str">
@@ -1211,6 +1231,9 @@
       <x:c r="T10" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U10" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="8" t="str">
@@ -1273,6 +1296,9 @@
       <x:c r="T11" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U11" s="10" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
       <x:c r="A12" s="8" t="str">
@@ -1335,6 +1361,9 @@
       <x:c r="T12" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U12" s="10" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
       <x:c r="A13" s="8" t="str">
@@ -1397,6 +1426,9 @@
       <x:c r="T13" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U13" s="10" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
       <x:c r="A14" s="8" t="str">
@@ -1459,6 +1491,9 @@
       <x:c r="T14" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U14" s="10" t="n">
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
       <x:c r="A15" s="8" t="str">
@@ -1521,6 +1556,9 @@
       <x:c r="T15" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U15" s="10" t="n">
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8" t="str">
@@ -1583,6 +1621,9 @@
       <x:c r="T16" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U16" s="10" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
@@ -1645,11 +1686,79 @@
       <x:c r="T17" s="10" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="U17" s="10" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="8" t="str">
+        <x:v>npc_dota_unit_undying_zombie</x:v>
+      </x:c>
+      <x:c r="B18" s="8" t="str">
+        <x:v>僵尸</x:v>
+      </x:c>
+      <x:c r="C18" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D18" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="9" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="F18" s="9" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="G18" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="9" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="I18" s="9" t="n">
+        <x:v>1600</x:v>
+      </x:c>
+      <x:c r="J18" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K18" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="L18" s="9" t="n">
+        <x:v>1300</x:v>
+      </x:c>
+      <x:c r="M18" s="9" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="N18" s="9" t="n">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="O18" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P18" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q18" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R18" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S18" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T18" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U18" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdde18527466d4d9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f177f1d4b534d88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2742,7 +2851,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7991a737ce434fbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e194fb5bc744bef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2920,10 +3029,32 @@
         <x:v>Wiki优先原生转身T=0.5；运行rad/s=T/0.03为平面匀速候选，不声称Dota加速度。基础攻速与BAT独立，buffer250。基础攻速100、后摇0为缺省候选；无攻击能力使攻击时钟无效。</x:v>
       </x:c>
     </x:row>
+    <x:row r="18" ht="64" customHeight="1">
+      <x:c r="A18" s="14" t="str">
+        <x:v>npc_dota_unit_undying_zombie</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C18" s="14" t="str">
+        <x:v>Native profile for Super zombie; one hero attack2HP/two ordinary attacks1HP. Raw .5/.03 follows the existing C4 unit-template conversion candidate, rather than silently introducing a second conversion. Backswing BAT-point=1.3 is explicit working animation value, not verified native animation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="64" customHeight="1">
+      <x:c r="A19" s="14" t="str">
+        <x:v>unit.Level</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>原生等级来自固定2023各单位自身Level字段，不按summoned标签一律当低级；远古/英雄型/幻象等技能资格仍由机制独立判断。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11ce1bb33d154360"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e9fef93b19e44c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint r6 C8: native action lifecycles, ice mechanics and 125 reviewed skills
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="Rb5b19717e0604f7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R1791269c7982447b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R00fe29731cf94c7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="Ra667aeb5d1e94c62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R182007c264484cf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R1a8173383ab14e12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R1e2e88ec21244aa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R09c821b5b93f40d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:U18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:U19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -198,7 +198,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>
@@ -735,7 +735,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59d2010013514261"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbebb325ddabf4c96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1755,10 +1755,75 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="8" t="str">
+        <x:v>npc_dota_item_wraith_pact_totem</x:v>
+      </x:c>
+      <x:c r="B19" s="8" t="str">
+        <x:v>怨灵图腾</x:v>
+      </x:c>
+      <x:c r="C19" s="9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="9" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="J19" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N19" s="9" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="O19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q19" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R19" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S19" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T19" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U19" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f177f1d4b534d88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a32739d14224d52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2851,7 +2916,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e194fb5bc744bef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a38836572c242ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3051,10 +3116,21 @@
         <x:v>原生等级来自固定2023各单位自身Level字段，不按summoned标签一律当低级；远古/英雄型/幻象等技能资格仍由机制独立判断。</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="64" customHeight="1">
+      <x:c r="A20" s="14" t="str">
+        <x:v>npc_dota_item_wraith_pact_totem</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>固定2023 npc_units模板及base继承：无攻击、Level0、8计数生命、150速度；turn .5/.03为现有平面匀速候选。2023Wiki4次英雄/8次非英雄攻击、25秒与来源归图腾；不声称原生转身加速度。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e9fef93b19e44c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37aac13ff00943d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint r6 C9: attack snapshots, native channels and 140 reviewed skills
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R182007c264484cf3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R1a8173383ab14e12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R1e2e88ec21244aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R09c821b5b93f40d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R96ad6533f8f742fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R0339a9d520904362"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="Rdfdaa8ab89294dbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R5cf4dcf4dd10485d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:U19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:U20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -198,7 +198,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>
@@ -735,7 +735,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbebb325ddabf4c96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1096dbb33fb43ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1820,10 +1820,75 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="8" t="str">
+        <x:v>npc_dota_zeus_cloud</x:v>
+      </x:c>
+      <x:c r="B20" s="8" t="str">
+        <x:v>雷云</x:v>
+      </x:c>
+      <x:c r="C20" s="9" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" s="9" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="J20" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K20" s="9" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="L20" s="9" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="M20" s="9" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="N20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P20" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q20" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R20" s="9" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="S20" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T20" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U20" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a32739d14224d52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c4fcd096e8b4e76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2916,7 +2981,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a38836572c242ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R169cc3a5d1a3423f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3127,10 +3192,21 @@
         <x:v>固定2023 npc_units模板及base继承：无攻击、Level0、8计数生命、150速度；turn .5/.03为现有平面匀速候选。2023Wiki4次英雄/8次非英雄攻击、25秒与来源归图腾；不声称原生转身加速度。</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="64" customHeight="1">
+      <x:c r="A21" s="14" t="str">
+        <x:v>npc_dota_zeus_cloud</x:v>
+      </x:c>
+      <x:c r="B21" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C21" s="14" t="str">
+        <x:v>2023 pinned npc_dota_zeus_cloud with base inherited fields; NO_ATTACK/ward profile. Source turn0.5/.03 remains C4candidate conversion, no actual attack claim.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37aac13ff00943d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a6a7a3bf6bb4b6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint r6 C10: typed attacks, native mana shield and 155 reviewed skills
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R96ad6533f8f742fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R0339a9d520904362"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="Rdfdaa8ab89294dbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R5cf4dcf4dd10485d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="Read31684637e4220"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="Rb0332d3230514087"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R61f7a858e92643b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R6d4323498ffc427c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:U20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:U22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -198,7 +198,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>
@@ -735,7 +735,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1096dbb33fb43ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26bb9a54b2644005"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1885,10 +1885,140 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="8" t="str">
+        <x:v>npc_dota_furion_treant_1</x:v>
+      </x:c>
+      <x:c r="B21" s="8" t="str">
+        <x:v>树人（原生1级）</x:v>
+      </x:c>
+      <x:c r="C21" s="9" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="9" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F21" s="9" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G21" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H21" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I21" s="9" t="n">
+        <x:v>1600</x:v>
+      </x:c>
+      <x:c r="J21" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K21" s="9" t="n">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="L21" s="9" t="n">
+        <x:v>533</x:v>
+      </x:c>
+      <x:c r="M21" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N21" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="O21" s="9" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="P21" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q21" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R21" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S21" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T21" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U21" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="8" t="str">
+        <x:v>npc_dota_furion_treant_2</x:v>
+      </x:c>
+      <x:c r="B22" s="8" t="str">
+        <x:v>树人（原生2级）</x:v>
+      </x:c>
+      <x:c r="C22" s="9" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="D22" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="9" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G22" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H22" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I22" s="9" t="n">
+        <x:v>1600</x:v>
+      </x:c>
+      <x:c r="J22" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K22" s="9" t="n">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="L22" s="9" t="n">
+        <x:v>533</x:v>
+      </x:c>
+      <x:c r="M22" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N22" s="9" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="O22" s="9" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="P22" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q22" s="9" t="n">
+        <x:v>83.33333333333334</x:v>
+      </x:c>
+      <x:c r="R22" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S22" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T22" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U22" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c4fcd096e8b4e76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8876b2aa35e408f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2981,7 +3111,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R169cc3a5d1a3423f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d15d3ee543e429a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3203,10 +3333,32 @@
         <x:v>2023 pinned npc_dota_zeus_cloud with base inherited fields; NO_ATTACK/ward profile. Source turn0.5/.03 remains C4candidate conversion, no actual attack claim.</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="64" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>npc_dota_furion_treant_1</x:v>
+      </x:c>
+      <x:c r="B22" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C22" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；AAHP/attack are explicit call overrides. Native profile1/2 is approved byroot. rawMovementTurnRate=0.5; profile2 raw2.5 conflicts generic oldWiki0.5; conversion remains existing C4candidate and source note must retain conflict. No unproved acceleration claim.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="64" customHeight="1">
+      <x:c r="A23" s="14" t="str">
+        <x:v>npc_dota_furion_treant_2</x:v>
+      </x:c>
+      <x:c r="B23" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C23" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；AAHP/attack are explicit call overrides. Native profile1/2 is approved byroot. rawMovementTurnRate=2.5; profile2 raw2.5 conflicts generic oldWiki0.5; conversion remains existing C4candidate and source note must retain conflict. No unproved acceleration claim.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a6a7a3bf6bb4b6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radb771c9c1874362"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Audit C11 skill mechanics, native attack classes and configuration
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="Read31684637e4220"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="Rb0332d3230514087"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R61f7a858e92643b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R6d4323498ffc427c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R5d29a8f88300436f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R534e586832eb462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R7591365c079a4ebc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R4b6f02daadff4623"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -83,7 +83,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -120,6 +120,9 @@
     <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -155,8 +158,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:U22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="21">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:X23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="24">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
     <x:tableColumn id="3" name="生命"/>
@@ -178,6 +181,9 @@
     <x:tableColumn id="19" name="攻击距离缓冲"/>
     <x:tableColumn id="20" name="攻击类型0无1近2远"/>
     <x:tableColumn id="21" name="原生等级"/>
+    <x:tableColumn id="22" name="穿刺对英雄倍率"/>
+    <x:tableColumn id="23" name="穿刺对普通单位倍率"/>
+    <x:tableColumn id="24" name="穿刺对强化防御倍率"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -198,7 +204,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>
@@ -735,7 +741,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26bb9a54b2644005"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e2b2a23d4b343b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -768,6 +774,9 @@
     <x:col min="19" max="19" width="17" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="22" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="15" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="22" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="22" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -844,6 +853,15 @@
       <x:c r="U4" s="7" t="str">
         <x:v>原生等级</x:v>
       </x:c>
+      <x:c r="V4" s="16" t="str">
+        <x:v>穿刺对英雄倍率</x:v>
+      </x:c>
+      <x:c r="W4" s="16" t="str">
+        <x:v>穿刺对普通单位倍率</x:v>
+      </x:c>
+      <x:c r="X4" s="16" t="str">
+        <x:v>穿刺对强化防御倍率</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="8" t="str">
@@ -909,6 +927,9 @@
       <x:c r="U5" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="V5" s="9"/>
+      <x:c r="W5" s="9"/>
+      <x:c r="X5" s="9"/>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
       <x:c r="A6" s="8" t="str">
@@ -974,6 +995,9 @@
       <x:c r="U6" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="V6" s="9"/>
+      <x:c r="W6" s="9"/>
+      <x:c r="X6" s="9"/>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="8" t="str">
@@ -1039,6 +1063,9 @@
       <x:c r="U7" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="V7" s="9"/>
+      <x:c r="W7" s="9"/>
+      <x:c r="X7" s="9"/>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="8" t="str">
@@ -1104,6 +1131,9 @@
       <x:c r="U8" s="10" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="V8" s="9"/>
+      <x:c r="W8" s="9"/>
+      <x:c r="X8" s="9"/>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="8" t="str">
@@ -1169,6 +1199,9 @@
       <x:c r="U9" s="10" t="n">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="V9" s="9"/>
+      <x:c r="W9" s="9"/>
+      <x:c r="X9" s="9"/>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="8" t="str">
@@ -1234,6 +1267,9 @@
       <x:c r="U10" s="10" t="n">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="V10" s="9"/>
+      <x:c r="W10" s="9"/>
+      <x:c r="X10" s="9"/>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="8" t="str">
@@ -1299,6 +1335,9 @@
       <x:c r="U11" s="10" t="n">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="V11" s="9"/>
+      <x:c r="W11" s="9"/>
+      <x:c r="X11" s="9"/>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
       <x:c r="A12" s="8" t="str">
@@ -1364,6 +1403,9 @@
       <x:c r="U12" s="10" t="n">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="V12" s="9"/>
+      <x:c r="W12" s="9"/>
+      <x:c r="X12" s="9"/>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
       <x:c r="A13" s="8" t="str">
@@ -1429,6 +1471,9 @@
       <x:c r="U13" s="10" t="n">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="V13" s="9"/>
+      <x:c r="W13" s="9"/>
+      <x:c r="X13" s="9"/>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
       <x:c r="A14" s="8" t="str">
@@ -1494,6 +1539,9 @@
       <x:c r="U14" s="10" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="V14" s="9"/>
+      <x:c r="W14" s="9"/>
+      <x:c r="X14" s="9"/>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
       <x:c r="A15" s="8" t="str">
@@ -1559,6 +1607,9 @@
       <x:c r="U15" s="10" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="V15" s="9"/>
+      <x:c r="W15" s="9"/>
+      <x:c r="X15" s="9"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8" t="str">
@@ -1624,6 +1675,9 @@
       <x:c r="U16" s="10" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="V16" s="9"/>
+      <x:c r="W16" s="9"/>
+      <x:c r="X16" s="9"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
@@ -1689,6 +1743,9 @@
       <x:c r="U17" s="10" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="V17" s="9"/>
+      <x:c r="W17" s="9"/>
+      <x:c r="X17" s="9"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8" t="str">
@@ -1754,6 +1811,9 @@
       <x:c r="U18" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="V18" s="9"/>
+      <x:c r="W18" s="9"/>
+      <x:c r="X18" s="9"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="8" t="str">
@@ -1819,6 +1879,9 @@
       <x:c r="U19" s="10" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="V19" s="9"/>
+      <x:c r="W19" s="9"/>
+      <x:c r="X19" s="9"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8" t="str">
@@ -1884,6 +1947,9 @@
       <x:c r="U20" s="10" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="V20" s="9"/>
+      <x:c r="W20" s="9"/>
+      <x:c r="X20" s="9"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="8" t="str">
@@ -1949,6 +2015,9 @@
       <x:c r="U21" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="V21" s="9"/>
+      <x:c r="W21" s="9"/>
+      <x:c r="X21" s="9"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="8" t="str">
@@ -2014,11 +2083,88 @@
       <x:c r="U22" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="V22" s="9"/>
+      <x:c r="W22" s="9"/>
+      <x:c r="X22" s="9"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="8" t="str">
+        <x:v>npc_dota_venomancer_plague_ward_1</x:v>
+      </x:c>
+      <x:c r="B23" s="8" t="str">
+        <x:v>瘟疫守卫（原生1级）</x:v>
+      </x:c>
+      <x:c r="C23" s="9" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="D23" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="9" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F23" s="9" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G23" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="9" t="n">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="J23" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K23" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="L23" s="9" t="n">
+        <x:v>1100</x:v>
+      </x:c>
+      <x:c r="M23" s="9" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="N23" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O23" s="9" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="P23" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q23" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R23" s="9" t="n">
+        <x:v>1900</x:v>
+      </x:c>
+      <x:c r="S23" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T23" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U23" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V23" s="9" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="W23" s="9" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="X23" s="9" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8876b2aa35e408f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddef1801e217482b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3111,7 +3257,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d15d3ee543e429a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceaf92e11dfc4561"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3355,10 +3501,21 @@
         <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；AAHP/attack are explicit call overrides. Native profile1/2 is approved byroot. rawMovementTurnRate=2.5; profile2 raw2.5 conflicts generic oldWiki0.5; conversion remains existing C4candidate and source note must retain conflict. No unproved acceleration claim.</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="64" customHeight="1">
+      <x:c r="A24" s="14" t="str">
+        <x:v>npc_dota_venomancer_plague_ward_1</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>20230216 KV ward1 identity; AA overrides HP/damage per five tiers. BaseAttackSpeed100 base-unit inherited. Back1.1 BAT-point engineering candidate; rawturn/.03 matches established project candidate.；原生模板不决定AA各档HP/攻击覆盖；pinned npc_units.txt11054原始攻击12至14；2023穿刺最终分类倍率：英雄0.5、普通单位1.5、强化防御0.35；https://web.archive.org/web/20230215192111id_/https://dota2.fandom.com/wiki/Attack_damage；空白表示不启用本分类，不给其它模板添加倍率。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radb771c9c1874362"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c89d1bdacc4ad9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify C12 contact timing motion and source attribution
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R5d29a8f88300436f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R534e586832eb462f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R7591365c079a4ebc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R4b6f02daadff4623"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R951e7d1ccd87448d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="Rb3b7959442534255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="Rdc02960cb47c48c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R0251fff7d4cd4437"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -158,7 +158,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:X23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:X24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="24">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -204,7 +204,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>
@@ -741,7 +741,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e2b2a23d4b343b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9339832243a645dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2161,10 +2161,78 @@
         <x:v>0.35</x:v>
       </x:c>
     </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="8" t="str">
+        <x:v>npc_dota_earth_spirit_stone</x:v>
+      </x:c>
+      <x:c r="B24" s="8" t="str">
+        <x:v>石之残岩</x:v>
+      </x:c>
+      <x:c r="C24" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="D24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="9" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="J24" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q24" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R24" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S24" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T24" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U24" s="10" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="V24" s="9"/>
+      <x:c r="W24" s="9"/>
+      <x:c r="X24" s="9"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddef1801e217482b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R979cfe42f3234e1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3257,7 +3325,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceaf92e11dfc4561"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb91951679034c28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3512,10 +3580,21 @@
         <x:v>20230216 KV ward1 identity; AA overrides HP/damage per five tiers. BaseAttackSpeed100 base-unit inherited. Back1.1 BAT-point engineering candidate; rawturn/.03 matches established project candidate.；原生模板不决定AA各档HP/攻击覆盖；pinned npc_units.txt11054原始攻击12至14；2023穿刺最终分类倍率：英雄0.5、普通单位1.5、强化防御0.35；https://web.archive.org/web/20230215192111id_/https://dota2.fandom.com/wiki/Attack_damage；空白表示不启用本分类，不给其它模板添加倍率。</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="64" customHeight="1">
+      <x:c r="A25" s="14" t="str">
+        <x:v>npc_dota_earth_spirit_stone</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原生自身HP100/Level4/无攻击/MS0；npc_dota_units_base继承Mana0/AS100/MR0/turn.5/buffer250；turn/.03沿既有平面候选，NO_ATTACK后摇0是工程候选非KV字段。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c89d1bdacc4ad9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51eb8fde0f504283"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify C13 restoration movement and native combat combinations
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -132,6 +132,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Config_units_0" displayName="Config_units_0" ref="A4:S8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:S8"/>
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="职业ID"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -159,6 +160,7 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:X24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:X24"/>
   <x:tableColumns count="24">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -191,6 +193,7 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Config_units_2" displayName="Config_units_2" ref="A4:F56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F56"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="组"/>
     <x:tableColumn id="2" name="字段"/>
@@ -205,6 +208,7 @@
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:C25"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>

</xml_diff>

<commit_message>
Verify C14 combat timing and summon lineage
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R951e7d1ccd87448d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="Rb3b7959442534255"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="Rdc02960cb47c48c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="R0251fff7d4cd4437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R8afbf4109e034aaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="Rf7172d87182a4d0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R35f88740a1e94016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="Rff7658392caa4d68"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -159,8 +159,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:X24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:X24"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:X34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:X34"/>
   <x:tableColumns count="24">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -207,8 +207,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:C25"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:C35"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>
@@ -745,7 +745,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9339832243a645dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R277951058d674497"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2233,10 +2233,690 @@
       <x:c r="W24" s="9"/>
       <x:c r="X24" s="9"/>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="8" t="str">
+        <x:v>npc_dota_visage_familiar1</x:v>
+      </x:c>
+      <x:c r="B25" s="8" t="str">
+        <x:v>佣兽1</x:v>
+      </x:c>
+      <x:c r="C25" s="9" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="D25" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E25" s="9" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F25" s="9" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G25" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H25" s="9" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="I25" s="9" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="J25" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K25" s="9" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="L25" s="9" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="M25" s="9" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="N25" s="9" t="n">
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="O25" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P25" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q25" s="9" t="n">
+        <x:v>30.000000000000004</x:v>
+      </x:c>
+      <x:c r="R25" s="9" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="S25" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T25" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U25" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="V25" s="9"/>
+      <x:c r="W25" s="9"/>
+      <x:c r="X25" s="9"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="8" t="str">
+        <x:v>npc_dota_visage_familiar2</x:v>
+      </x:c>
+      <x:c r="B26" s="8" t="str">
+        <x:v>佣兽2</x:v>
+      </x:c>
+      <x:c r="C26" s="9" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="D26" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E26" s="9" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F26" s="9" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G26" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H26" s="9" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="I26" s="9" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="J26" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K26" s="9" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="L26" s="9" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="M26" s="9" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="N26" s="9" t="n">
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="O26" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P26" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q26" s="9" t="n">
+        <x:v>30.000000000000004</x:v>
+      </x:c>
+      <x:c r="R26" s="9" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="S26" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T26" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U26" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="V26" s="9"/>
+      <x:c r="W26" s="9"/>
+      <x:c r="X26" s="9"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="8" t="str">
+        <x:v>npc_dota_visage_familiar3</x:v>
+      </x:c>
+      <x:c r="B27" s="8" t="str">
+        <x:v>佣兽3</x:v>
+      </x:c>
+      <x:c r="C27" s="9" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="D27" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="9" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="F27" s="9" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="G27" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H27" s="9" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="I27" s="9" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="J27" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K27" s="9" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="L27" s="9" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="M27" s="9" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="N27" s="9" t="n">
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="O27" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P27" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q27" s="9" t="n">
+        <x:v>30.000000000000004</x:v>
+      </x:c>
+      <x:c r="R27" s="9" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="S27" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T27" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U27" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="V27" s="9"/>
+      <x:c r="W27" s="9"/>
+      <x:c r="X27" s="9"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="8" t="str">
+        <x:v>npc_dota_lone_druid_bear1</x:v>
+      </x:c>
+      <x:c r="B28" s="8" t="str">
+        <x:v>灵熊1</x:v>
+      </x:c>
+      <x:c r="C28" s="9" t="n">
+        <x:v>1100</x:v>
+      </x:c>
+      <x:c r="D28" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="E28" s="9" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="F28" s="9" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G28" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H28" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I28" s="9" t="n">
+        <x:v>1750</x:v>
+      </x:c>
+      <x:c r="J28" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K28" s="9" t="n">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="L28" s="9" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="M28" s="9" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="N28" s="9" t="n">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="O28" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="P28" s="9" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="Q28" s="9" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R28" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S28" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T28" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U28" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V28" s="9"/>
+      <x:c r="W28" s="9"/>
+      <x:c r="X28" s="9"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="8" t="str">
+        <x:v>npc_dota_lone_druid_bear2</x:v>
+      </x:c>
+      <x:c r="B29" s="8" t="str">
+        <x:v>灵熊2</x:v>
+      </x:c>
+      <x:c r="C29" s="9" t="n">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="D29" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="E29" s="9" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="F29" s="9" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G29" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H29" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I29" s="9" t="n">
+        <x:v>1650</x:v>
+      </x:c>
+      <x:c r="J29" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K29" s="9" t="n">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="L29" s="9" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="M29" s="9" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="N29" s="9" t="n">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="O29" s="9" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="P29" s="9" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="Q29" s="9" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R29" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S29" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T29" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U29" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V29" s="9"/>
+      <x:c r="W29" s="9"/>
+      <x:c r="X29" s="9"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="8" t="str">
+        <x:v>npc_dota_lone_druid_bear4</x:v>
+      </x:c>
+      <x:c r="B30" s="8" t="str">
+        <x:v>灵熊4</x:v>
+      </x:c>
+      <x:c r="C30" s="9" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D30" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="E30" s="9" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="F30" s="9" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G30" s="9" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H30" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" s="9" t="n">
+        <x:v>1450</x:v>
+      </x:c>
+      <x:c r="J30" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K30" s="9" t="n">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="L30" s="9" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="M30" s="9" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="N30" s="9" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="O30" s="9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="P30" s="9" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="Q30" s="9" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R30" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S30" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T30" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U30" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V30" s="9"/>
+      <x:c r="W30" s="9"/>
+      <x:c r="X30" s="9"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="8" t="str">
+        <x:v>npc_dota_lycan_wolf1</x:v>
+      </x:c>
+      <x:c r="B31" s="8" t="str">
+        <x:v>狼1</x:v>
+      </x:c>
+      <x:c r="C31" s="9" t="n">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="D31" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E31" s="9" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F31" s="9" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G31" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H31" s="9" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="I31" s="9" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="J31" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K31" s="9" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="L31" s="9" t="n">
+        <x:v>640</x:v>
+      </x:c>
+      <x:c r="M31" s="9" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="N31" s="9" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="O31" s="9" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="P31" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q31" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R31" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S31" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T31" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U31" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V31" s="9"/>
+      <x:c r="W31" s="9"/>
+      <x:c r="X31" s="9"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="8" t="str">
+        <x:v>npc_dota_lycan_wolf2</x:v>
+      </x:c>
+      <x:c r="B32" s="8" t="str">
+        <x:v>狼2</x:v>
+      </x:c>
+      <x:c r="C32" s="9" t="n">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="D32" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E32" s="9" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F32" s="9" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="G32" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H32" s="9" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="I32" s="9" t="n">
+        <x:v>1100</x:v>
+      </x:c>
+      <x:c r="J32" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K32" s="9" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="L32" s="9" t="n">
+        <x:v>640</x:v>
+      </x:c>
+      <x:c r="M32" s="9" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="N32" s="9" t="n">
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="O32" s="9" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="P32" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q32" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R32" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S32" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T32" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U32" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="V32" s="9"/>
+      <x:c r="W32" s="9"/>
+      <x:c r="X32" s="9"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="8" t="str">
+        <x:v>npc_dota_wraith_king_skeleton_warrior</x:v>
+      </x:c>
+      <x:c r="B33" s="8" t="str">
+        <x:v>骷髅战士</x:v>
+      </x:c>
+      <x:c r="C33" s="9" t="n">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="D33" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E33" s="9" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F33" s="9" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="G33" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H33" s="9" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="I33" s="9" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="J33" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K33" s="9" t="n">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="L33" s="9" t="n">
+        <x:v>640</x:v>
+      </x:c>
+      <x:c r="M33" s="9" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="N33" s="9" t="n">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="O33" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P33" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q33" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R33" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S33" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T33" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U33" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V33" s="9"/>
+      <x:c r="W33" s="9"/>
+      <x:c r="X33" s="9"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="8" t="str">
+        <x:v>npc_dota_clinkz_skeleton_archer</x:v>
+      </x:c>
+      <x:c r="B34" s="8" t="str">
+        <x:v>骷髅射手</x:v>
+      </x:c>
+      <x:c r="C34" s="9" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="D34" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E34" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F34" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G34" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H34" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" s="9" t="n">
+        <x:v>1600</x:v>
+      </x:c>
+      <x:c r="J34" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K34" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="L34" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M34" s="9" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="N34" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O34" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P34" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q34" s="9" t="n">
+        <x:v>16.666666666666668</x:v>
+      </x:c>
+      <x:c r="R34" s="9" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="S34" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T34" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U34" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V34" s="9"/>
+      <x:c r="W34" s="9"/>
+      <x:c r="X34" s="9"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R979cfe42f3234e1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R300182be35a44f53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3329,7 +4009,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb91951679034c28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34330b78033a4f1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3595,10 +4275,120 @@
         <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原生自身HP100/Level4/无攻击/MS0；npc_dota_units_base继承Mana0/AS100/MR0/turn.5/buffer250；turn/.03沿既有平面候选，NO_ATTACK后摇0是工程候选非KV字段。</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="64" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>npc_dota_visage_familiar1</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原始KV独立单位模板；动画点/后摇取具名保留Wiki，灵熊与骷髅来自2023直接页；turn/0.03为平面匀速换算候选。AA父技能独立覆盖明确数值，未修改旧20模板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="64" customHeight="1">
+      <x:c r="A27" s="14" t="str">
+        <x:v>npc_dota_visage_familiar2</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C27" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原始KV独立单位模板；动画点/后摇取具名保留Wiki，灵熊与骷髅来自2023直接页；turn/0.03为平面匀速换算候选。AA父技能独立覆盖明确数值，未修改旧20模板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="64" customHeight="1">
+      <x:c r="A28" s="14" t="str">
+        <x:v>npc_dota_visage_familiar3</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原始KV独立单位模板；动画点/后摇取具名保留Wiki，灵熊与骷髅来自2023直接页；turn/0.03为平面匀速换算候选。AA父技能独立覆盖明确数值，未修改旧20模板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="64" customHeight="1">
+      <x:c r="A29" s="14" t="str">
+        <x:v>npc_dota_lone_druid_bear1</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C29" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原始KV独立单位模板；动画点/后摇取具名保留Wiki，灵熊与骷髅来自2023直接页；turn/0.03为平面匀速换算候选。AA父技能独立覆盖明确数值，未修改旧20模板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="64" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>npc_dota_lone_druid_bear2</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原始KV独立单位模板；动画点/后摇取具名保留Wiki，灵熊与骷髅来自2023直接页；turn/0.03为平面匀速换算候选。AA父技能独立覆盖明确数值，未修改旧20模板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="64" customHeight="1">
+      <x:c r="A31" s="14" t="str">
+        <x:v>npc_dota_lone_druid_bear4</x:v>
+      </x:c>
+      <x:c r="B31" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C31" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原始KV独立单位模板；动画点/后摇取具名保留Wiki，灵熊与骷髅来自2023直接页；turn/0.03为平面匀速换算候选。AA父技能独立覆盖明确数值，未修改旧20模板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="64" customHeight="1">
+      <x:c r="A32" s="14" t="str">
+        <x:v>npc_dota_lycan_wolf1</x:v>
+      </x:c>
+      <x:c r="B32" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原始KV独立单位模板；动画点/后摇取具名保留Wiki，灵熊与骷髅来自2023直接页；turn/0.03为平面匀速换算候选。AA父技能独立覆盖明确数值，未修改旧20模板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="64" customHeight="1">
+      <x:c r="A33" s="14" t="str">
+        <x:v>npc_dota_lycan_wolf2</x:v>
+      </x:c>
+      <x:c r="B33" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C33" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原始KV独立单位模板；动画点/后摇取具名保留Wiki，灵熊与骷髅来自2023直接页；turn/0.03为平面匀速换算候选。AA父技能独立覆盖明确数值，未修改旧20模板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="64" customHeight="1">
+      <x:c r="A34" s="14" t="str">
+        <x:v>npc_dota_wraith_king_skeleton_warrior</x:v>
+      </x:c>
+      <x:c r="B34" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；原始KV独立单位模板；动画点/后摇取具名保留Wiki，灵熊与骷髅来自2023直接页；turn/0.03为平面匀速换算候选。AA父技能独立覆盖明确数值，未修改旧20模板。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="64" customHeight="1">
+      <x:c r="A35" s="14" t="str">
+        <x:v>npc_dota_clinkz_skeleton_archer</x:v>
+      </x:c>
+      <x:c r="B35" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C35" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；Pinned20230210npc unit rawBAT1.7,abilityattack_rate1.6overrides;tablekeepssinglefinaleffective1.6.LPFandom20230215AP/back.3+.3/projectile900/rawturn.5/HP1000;BaseAS100/buffer250frombaseunitinheritance.No changes to20oldtemplates.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51eb8fde0f504283"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e3ad21d89534a29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implement C15 combat timing and settlement corrections
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="R8afbf4109e034aaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="Rf7172d87182a4d0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R35f88740a1e94016"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="Rff7658392caa4d68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="Rbc0a21a5e8c849d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R38c4108548ec4a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R3a664b5911f74a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="Rd26713c866c74a93"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -159,8 +159,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:X34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:X34"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Config_units_1" displayName="Config_units_1" ref="A4:X37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:X37"/>
   <x:tableColumns count="24">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="中文名称"/>
@@ -207,8 +207,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:C35"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:C38"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>
@@ -745,7 +745,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R277951058d674497"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R770f9cd8cfe44aab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2913,10 +2913,214 @@
       <x:c r="W34" s="9"/>
       <x:c r="X34" s="9"/>
     </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="8" t="str">
+        <x:v>npc_dota_beastmaster_boar</x:v>
+      </x:c>
+      <x:c r="B35" s="8" t="str">
+        <x:v>豪猪</x:v>
+      </x:c>
+      <x:c r="C35" s="9" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="D35" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="9" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F35" s="9" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G35" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H35" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I35" s="9" t="n">
+        <x:v>1250</x:v>
+      </x:c>
+      <x:c r="J35" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K35" s="9" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="L35" s="9" t="n">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="M35" s="9" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="N35" s="9" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="O35" s="9" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="P35" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q35" s="9" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="R35" s="9" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="S35" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T35" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U35" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V35" s="9"/>
+      <x:c r="W35" s="9"/>
+      <x:c r="X35" s="9"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="8" t="str">
+        <x:v>npc_dota_warlock_golem</x:v>
+      </x:c>
+      <x:c r="B36" s="8" t="str">
+        <x:v>地狱火</x:v>
+      </x:c>
+      <x:c r="C36" s="9" t="n">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="D36" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E36" s="9" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="F36" s="9" t="n">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="G36" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H36" s="9" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="I36" s="9" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="J36" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K36" s="9" t="n">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="L36" s="9" t="n">
+        <x:v>570</x:v>
+      </x:c>
+      <x:c r="M36" s="9" t="n">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="N36" s="9" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="O36" s="9" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="P36" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q36" s="9" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="R36" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S36" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T36" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U36" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V36" s="9"/>
+      <x:c r="W36" s="9"/>
+      <x:c r="X36" s="9"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="8" t="str">
+        <x:v>npc_dota_phoenix_sun</x:v>
+      </x:c>
+      <x:c r="B37" s="8" t="str">
+        <x:v>超新星烈日</x:v>
+      </x:c>
+      <x:c r="C37" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="D37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I37" s="9" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="J37" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q37" s="9" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="R37" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S37" s="9" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T37" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U37" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V37" s="9"/>
+      <x:c r="W37" s="9"/>
+      <x:c r="X37" s="9"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R300182be35a44f53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8521a1524ee4b6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4009,7 +4213,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34330b78033a4f1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36327b0aa1e34a39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4385,10 +4589,43 @@
         <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；Pinned20230210npc unit rawBAT1.7,abilityattack_rate1.6overrides;tablekeepssinglefinaleffective1.6.LPFandom20230215AP/back.3+.3/projectile900/rawturn.5/HP1000;BaseAS100/buffer250frombaseunitinheritance.No changes to20oldtemplates.</x:v>
       </x:c>
     </x:row>
+    <x:row r="36" ht="64" customHeight="1">
+      <x:c r="A36" s="14" t="str">
+        <x:v>npc_dota_beastmaster_boar</x:v>
+      </x:c>
+      <x:c r="B36" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C36" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；Identity only; preserve AA HP/damage/armor/BAT/range/movement/abilities.；Boar explicit turn.6; Golem inherits base.5; both resolved directly from pinned KV. Engine angular conversion x30 remains working model.；Backswing native Wiki.5+.47 and.26+.57; retained pre-C15 working values; precise original AA animation unknown.；Only generic pinned unit IDs exist; do not fabricate numbered variants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="64" customHeight="1">
+      <x:c r="A37" s="14" t="str">
+        <x:v>npc_dota_warlock_golem</x:v>
+      </x:c>
+      <x:c r="B37" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C37" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；Identity only; preserve AA HP/damage/armor/BAT/range/movement/abilities.；Boar explicit turn.6; Golem inherits base.5; both resolved directly from pinned KV. Engine angular conversion x30 remains working model.；Backswing native Wiki.5+.47 and.26+.57; retained pre-C15 working values; precise original AA animation unknown.；Only generic pinned unit IDs exist; do not fabricate numbered variants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="64" customHeight="1">
+      <x:c r="A38" s="14" t="str">
+        <x:v>npc_dota_phoenix_sun</x:v>
+      </x:c>
+      <x:c r="B38" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt</x:v>
+      </x:c>
+      <x:c r="C38" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；Raw native additive ward body:100HP/0attack/NONE move;BaseAttackSpeed100/turn18/mana0 are nonacting engineering defaults where the raw block omits values. Hit-count class/tier semantics are ability parameters,not fake HP.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e3ad21d89534a29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0484166664f54094"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Release v0.1.1-r7: shop clarity and round-based hero growth
</commit_message>
<xml_diff>
--- a/config/单位配置.xlsx
+++ b/config/单位配置.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="Rbc0a21a5e8c849d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="R38c4108548ec4a14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="R3a664b5911f74a54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="Rd26713c866c74a93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="职业" sheetId="1" r:id="Rb724d2ef7a834737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="召唤单位" sheetId="2" r:id="Rb53779899141406c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="底层规则" sheetId="3" r:id="Rcba37b926f574864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原生单位来源" sheetId="4" r:id="Rcb70e7c9caff424d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -83,7 +83,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -123,6 +123,9 @@
     <x:xf numFmtId="200" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -131,28 +134,31 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Config_units_0" displayName="Config_units_0" ref="A4:S8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:S8"/>
-  <x:tableColumns count="19">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Config_units_0" displayName="Config_units_0" ref="A4:V8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:V8"/>
+  <x:tableColumns count="22">
     <x:tableColumn id="1" name="职业ID"/>
     <x:tableColumn id="2" name="中文名称"/>
     <x:tableColumn id="3" name="颜色"/>
-    <x:tableColumn id="4" name="生命"/>
-    <x:tableColumn id="5" name="法力"/>
-    <x:tableColumn id="6" name="攻击"/>
-    <x:tableColumn id="7" name="护甲"/>
+    <x:tableColumn id="4" name="1级完整生命（已含基础属性）"/>
+    <x:tableColumn id="5" name="1级完整法力（已含基础属性）"/>
+    <x:tableColumn id="6" name="1级完整攻击（已含基础属性）"/>
+    <x:tableColumn id="7" name="1级完整护甲（已含基础属性）"/>
     <x:tableColumn id="8" name="攻击间隔ms"/>
     <x:tableColumn id="9" name="攻击距离"/>
     <x:tableColumn id="10" name="移动速度"/>
-    <x:tableColumn id="11" name="力量"/>
-    <x:tableColumn id="12" name="敏捷"/>
-    <x:tableColumn id="13" name="智力"/>
+    <x:tableColumn id="11" name="1级力量"/>
+    <x:tableColumn id="12" name="1级敏捷"/>
+    <x:tableColumn id="13" name="1级智力"/>
     <x:tableColumn id="14" name="主属性"/>
     <x:tableColumn id="15" name="转身速度rad每秒"/>
     <x:tableColumn id="16" name="攻击前摇ms"/>
     <x:tableColumn id="17" name="攻击后摇ms"/>
     <x:tableColumn id="18" name="弹体速度"/>
     <x:tableColumn id="19" name="攻击距离缓冲"/>
+    <x:tableColumn id="20" name="每级力量成长"/>
+    <x:tableColumn id="21" name="每级敏捷成长"/>
+    <x:tableColumn id="22" name="每级智力成长"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -207,8 +213,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:C38"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Native_Profile_Sources" displayName="Native_Profile_Sources" ref="A4:C42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:C42"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="单位ID"/>
     <x:tableColumn id="2" name="来源"/>
@@ -435,6 +441,9 @@
     <x:col min="17" max="17" width="17" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="17" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -444,10 +453,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>四职业男女同属性。生命、法力、攻击已含基础属性，勿再次全量叠加。转身18rad/s、攻击点及缓冲为项目工作值。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="26" customHeight="1">
+        <x:v>D:G为1级完整值（已含基础属性），K:M为1级基础三围；T:V为每级属性点成长，不是直接生命/法力成长。初始攻速保留项目100基准。动作、射程、移动及转身保持项目工作值；原生来源与换算见“原生单位来源”。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="7" t="str">
         <x:v>职业ID</x:v>
       </x:c>
@@ -457,17 +466,17 @@
       <x:c r="C4" s="7" t="str">
         <x:v>颜色</x:v>
       </x:c>
-      <x:c r="D4" s="7" t="str">
-        <x:v>生命</x:v>
-      </x:c>
-      <x:c r="E4" s="7" t="str">
-        <x:v>法力</x:v>
-      </x:c>
-      <x:c r="F4" s="7" t="str">
-        <x:v>攻击</x:v>
-      </x:c>
-      <x:c r="G4" s="7" t="str">
-        <x:v>护甲</x:v>
+      <x:c r="D4" s="17" t="str">
+        <x:v>1级完整生命（已含基础属性）</x:v>
+      </x:c>
+      <x:c r="E4" s="17" t="str">
+        <x:v>1级完整法力（已含基础属性）</x:v>
+      </x:c>
+      <x:c r="F4" s="17" t="str">
+        <x:v>1级完整攻击（已含基础属性）</x:v>
+      </x:c>
+      <x:c r="G4" s="17" t="str">
+        <x:v>1级完整护甲（已含基础属性）</x:v>
       </x:c>
       <x:c r="H4" s="7" t="str">
         <x:v>攻击间隔ms</x:v>
@@ -479,13 +488,13 @@
         <x:v>移动速度</x:v>
       </x:c>
       <x:c r="K4" s="7" t="str">
-        <x:v>力量</x:v>
+        <x:v>1级力量</x:v>
       </x:c>
       <x:c r="L4" s="7" t="str">
-        <x:v>敏捷</x:v>
+        <x:v>1级敏捷</x:v>
       </x:c>
       <x:c r="M4" s="7" t="str">
-        <x:v>智力</x:v>
+        <x:v>1级智力</x:v>
       </x:c>
       <x:c r="N4" s="7" t="str">
         <x:v>主属性</x:v>
@@ -504,6 +513,15 @@
       </x:c>
       <x:c r="S4" s="7" t="str">
         <x:v>攻击距离缓冲</x:v>
+      </x:c>
+      <x:c r="T4" s="7" t="str">
+        <x:v>每级力量成长</x:v>
+      </x:c>
+      <x:c r="U4" s="7" t="str">
+        <x:v>每级敏捷成长</x:v>
+      </x:c>
+      <x:c r="V4" s="7" t="str">
+        <x:v>每级智力成长</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
@@ -517,16 +535,16 @@
         <x:v>#20c9d8</x:v>
       </x:c>
       <x:c r="D5" s="9" t="n">
-        <x:v>1050</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="E5" s="9" t="n">
-        <x:v>550</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>52.5</x:v>
       </x:c>
       <x:c r="G5" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>3.34</x:v>
       </x:c>
       <x:c r="H5" s="9" t="n">
         <x:v>1450</x:v>
@@ -538,13 +556,13 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="K5" s="9" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="L5" s="9" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="L5" s="9" t="n">
-        <x:v>30</x:v>
-      </x:c>
       <x:c r="M5" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="N5" s="9" t="str">
         <x:v>agility</x:v>
@@ -563,6 +581,15 @@
       </x:c>
       <x:c r="S5" s="9" t="n">
         <x:v>50</x:v>
+      </x:c>
+      <x:c r="T5" s="9" t="n">
+        <x:v>1.9</x:v>
+      </x:c>
+      <x:c r="U5" s="9" t="n">
+        <x:v>2.9</x:v>
+      </x:c>
+      <x:c r="V5" s="9" t="n">
+        <x:v>1.4</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -576,16 +603,16 @@
         <x:v>#ee3f68</x:v>
       </x:c>
       <x:c r="D6" s="9" t="n">
-        <x:v>1350</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="E6" s="9" t="n">
-        <x:v>500</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="F6" s="9" t="n">
-        <x:v>100</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="G6" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>4.841</x:v>
       </x:c>
       <x:c r="H6" s="9" t="n">
         <x:v>1250</x:v>
@@ -597,13 +624,13 @@
         <x:v>380</x:v>
       </x:c>
       <x:c r="K6" s="9" t="n">
-        <x:v>24</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="L6" s="9" t="n">
-        <x:v>28</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="M6" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="N6" s="9" t="str">
         <x:v>agility</x:v>
@@ -622,6 +649,15 @@
       </x:c>
       <x:c r="S6" s="9" t="n">
         <x:v>50</x:v>
+      </x:c>
+      <x:c r="T6" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U6" s="9" t="n">
+        <x:v>3.2</x:v>
+      </x:c>
+      <x:c r="V6" s="9" t="n">
+        <x:v>1.4</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
@@ -635,16 +671,16 @@
         <x:v>#9775f2</x:v>
       </x:c>
       <x:c r="D7" s="9" t="n">
-        <x:v>1000</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="E7" s="9" t="n">
-        <x:v>1000</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="F7" s="9" t="n">
-        <x:v>65</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="G7" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>1.672</x:v>
       </x:c>
       <x:c r="H7" s="9" t="n">
         <x:v>1700</x:v>
@@ -656,13 +692,13 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="K7" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="L7" s="9" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="M7" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="N7" s="9" t="str">
         <x:v>intelligence</x:v>
@@ -681,6 +717,15 @@
       </x:c>
       <x:c r="S7" s="9" t="n">
         <x:v>50</x:v>
+      </x:c>
+      <x:c r="T7" s="9" t="n">
+        <x:v>2.2</x:v>
+      </x:c>
+      <x:c r="U7" s="9" t="n">
+        <x:v>1.6</x:v>
+      </x:c>
+      <x:c r="V7" s="9" t="n">
+        <x:v>3.3</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
@@ -694,16 +739,16 @@
         <x:v>#efb83e</x:v>
       </x:c>
       <x:c r="D8" s="9" t="n">
-        <x:v>2100</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="E8" s="9" t="n">
-        <x:v>500</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>75</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="G8" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>0.505</x:v>
       </x:c>
       <x:c r="H8" s="9" t="n">
         <x:v>1800</x:v>
@@ -715,13 +760,13 @@
         <x:v>270</x:v>
       </x:c>
       <x:c r="K8" s="9" t="n">
-        <x:v>32</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="L8" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="M8" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="N8" s="9" t="str">
         <x:v>strength</x:v>
@@ -740,12 +785,21 @@
       </x:c>
       <x:c r="S8" s="9" t="n">
         <x:v>50</x:v>
+      </x:c>
+      <x:c r="T8" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="U8" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V8" s="9" t="n">
+        <x:v>1.6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R770f9cd8cfe44aab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd3b66aa91c741d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3120,7 +3174,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8521a1524ee4b6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b35521490bc4222"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4213,7 +4267,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36327b0aa1e34a39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd15933d86aa84b9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4234,7 +4288,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>数值权威在“召唤单位”；本页仅说明来源与候选换算，不提供另一份可编辑副本。</x:v>
+        <x:v>“召唤单位”和“职业”为数值权威；本页仅说明来源与候选换算，不提供另一份可编辑副本。职业1级完整值已含基础属性，每级成长是独立属性点。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
@@ -4622,10 +4676,54 @@
         <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_units.txt；Raw native additive ward body:100HP/0attack/NONE move;BaseAttackSpeed100/turn18/mana0 are nonacting engineering defaults where the raw block omits values. Hit-count class/tier semantics are ability parameters,not fake HP.</x:v>
       </x:c>
     </x:row>
+    <x:row r="39" ht="100" customHeight="1">
+      <x:c r="A39" s="14" t="str">
+        <x:v>role:assassin</x:v>
+      </x:c>
+      <x:c r="B39" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_heroes.txt</x:v>
+      </x:c>
+      <x:c r="C39" s="14" t="str">
+        <x:v>2023-02-10固定KV，模板npc_dota_hero_phantom_assassin。基HP200+力量×22=618；基MP75+智力×12=255；原生攻击均值(31+33)/2+主属性=55；原生基础护甲1+敏捷×0.167=4.841。三围成长2/3.2/1.4属性点/级。仅L1完整值与成长可编辑；原始量只作来源说明。初始AS100及动作/移动/射程保持项目自定义，不引入模板原生AS。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="100" customHeight="1">
+      <x:c r="A40" s="14" t="str">
+        <x:v>role:archer</x:v>
+      </x:c>
+      <x:c r="B40" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_heroes.txt</x:v>
+      </x:c>
+      <x:c r="C40" s="14" t="str">
+        <x:v>2023-02-10固定KV，模板npc_dota_hero_drow_ranger。基HP200+力量×22=552；基MP75+智力×12=255；原生攻击均值(29+36)/2+主属性=52.5；原生基础护甲0+敏捷×0.167=3.34。三围成长1.9/2.9/1.4属性点/级。仅L1完整值与成长可编辑；原始量只作来源说明。初始AS100及动作/移动/射程保持项目自定义，不引入模板原生AS。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="100" customHeight="1">
+      <x:c r="A41" s="14" t="str">
+        <x:v>role:mage</x:v>
+      </x:c>
+      <x:c r="B41" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_heroes.txt</x:v>
+      </x:c>
+      <x:c r="C41" s="14" t="str">
+        <x:v>2023-02-10固定KV，模板npc_dota_hero_crystal_maiden。基HP200+力量×22=574；基MP75+智力×12=267；原生攻击均值(28+34)/2+主属性=47；原生基础护甲-1+敏捷×0.167=1.672。三围成长2.2/1.6/3.3属性点/级。仅L1完整值与成长可编辑；原始量只作来源说明。初始AS100及动作/移动/射程保持项目自定义，不引入模板原生AS。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="100" customHeight="1">
+      <x:c r="A42" s="14" t="str">
+        <x:v>role:tank</x:v>
+      </x:c>
+      <x:c r="B42" s="14" t="str">
+        <x:v>https://github.com/SteamTracking/GameTracking-Dota2/blob/6abdd9d13de2f4330ca748082467b9ff6e6cd928/game/dota/pak01_dir/scripts/npc/npc_heroes.txt</x:v>
+      </x:c>
+      <x:c r="C42" s="14" t="str">
+        <x:v>2023-02-10固定KV，模板npc_dota_hero_centaur。基HP200+力量×22=794；基MP75+智力×12=255；原生攻击均值(36+38)/2+主属性=64；原生基础护甲-2+敏捷×0.167=0.505。三围成长4/1/1.6属性点/级。仅L1完整值与成长可编辑；原始量只作来源说明。初始AS100及动作/移动/射程保持项目自定义，不引入模板原生AS。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0484166664f54094"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1de0404a1e83409f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>